<commit_message>
missing 999 for SM + SF
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/agegroups/AgeGroups_2025-06.xlsx
+++ b/owlcms/src/main/resources/agegroups/AgeGroups_2025-06.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\agegroups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB18353-63C4-42CC-9BD3-F86E967A9CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33347C83-8180-49D8-91EA-F1DDE3B9F1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2430" yWindow="2685" windowWidth="24615" windowHeight="11310" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="77">
   <si>
     <t>code</t>
   </si>
@@ -706,7 +706,9 @@
       <c r="H2" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="6"/>
+      <c r="J2" s="6" t="s">
+        <v>51</v>
+      </c>
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
@@ -2000,7 +2002,9 @@
       <c r="H25" t="s">
         <v>76</v>
       </c>
-      <c r="J25" s="6"/>
+      <c r="J25" s="6" t="s">
+        <v>51</v>
+      </c>
       <c r="K25" s="6"/>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>

</xml_diff>

<commit_message>
spurious JR F 999 categ
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/agegroups/AgeGroups_2025-06.xlsx
+++ b/owlcms/src/main/resources/agegroups/AgeGroups_2025-06.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\agegroups\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\agegroups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33347C83-8180-49D8-91EA-F1DDE3B9F1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C90DDA-103E-4AC6-B8E8-597BBF908DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="77">
   <si>
     <t>code</t>
   </si>
@@ -1851,9 +1851,7 @@
       <c r="R22" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="S22" s="6" t="s">
-        <v>51</v>
-      </c>
+      <c r="S22" s="6"/>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>

</xml_diff>

<commit_message>
Fix: Missing 2025 body weight category for female JR heavyweights
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/agegroups/AgeGroups_2025-06.xlsx
+++ b/owlcms/src/main/resources/agegroups/AgeGroups_2025-06.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\agegroups\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms4\owlcms\src\main\resources\agegroups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C90DDA-103E-4AC6-B8E8-597BBF908DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6269CFD-6BB3-4430-A5D3-1E352A846FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="77">
   <si>
     <t>code</t>
   </si>
@@ -1849,9 +1849,11 @@
         <v>59</v>
       </c>
       <c r="R22" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="S22" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="S22" s="6" t="s">
+        <v>51</v>
+      </c>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>

</xml_diff>